<commit_message>
fix: diagnóstico sync + tipos documento + cliente_nome opcional
</commit_message>
<xml_diff>
--- a/frontend/public/template-faturas.xlsx
+++ b/frontend/public/template-faturas.xlsx
@@ -397,17 +397,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:H5"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="28.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -418,24 +417,21 @@
         <v>cliente_codigo</v>
       </c>
       <c r="C1" t="str">
-        <v>cliente_nome</v>
+        <v>tipo_documento</v>
       </c>
       <c r="D1" t="str">
-        <v>tipo_documento</v>
+        <v>artigo_ref</v>
       </c>
       <c r="E1" t="str">
-        <v>artigo_ref</v>
+        <v>quantidade</v>
       </c>
       <c r="F1" t="str">
-        <v>quantidade</v>
+        <v>preco_unitario</v>
       </c>
       <c r="G1" t="str">
-        <v>preco_unitario</v>
+        <v>desconto_pct</v>
       </c>
       <c r="H1" t="str">
-        <v>desconto_pct</v>
-      </c>
-      <c r="I1" t="str">
         <v>comentario</v>
       </c>
     </row>
@@ -447,26 +443,22 @@
         <v>82</v>
       </c>
       <c r="C2" t="str">
-        <v>PRESTIMA SL Sucursal</v>
+        <v>FAA</v>
       </c>
       <c r="D2" t="str">
-        <v>FAA</v>
-      </c>
-      <c r="E2" t="str">
         <v>SERV REB</v>
       </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
       <c r="F2">
-        <v>1</v>
+        <v>150</v>
       </c>
       <c r="G2">
-        <v>150</v>
-      </c>
-      <c r="H2">
         <v>0</v>
       </c>
-      <c r="I2" t="str" xml:space="preserve">
+      <c r="H2" t="str" xml:space="preserve">
         <v xml:space="preserve">MARCA: Toyota
-MODELO: Yaris
 MATRICULA: 00-AA-00</v>
       </c>
     </row>
@@ -478,24 +470,21 @@
         <v>82</v>
       </c>
       <c r="C3" t="str">
-        <v>PRESTIMA SL Sucursal</v>
+        <v>FAA</v>
       </c>
       <c r="D3" t="str">
-        <v>FAA</v>
-      </c>
-      <c r="E3" t="str">
         <v>SERV MEC</v>
       </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
       <c r="F3">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="G3">
-        <v>80</v>
-      </c>
-      <c r="H3">
         <v>0</v>
       </c>
-      <c r="I3" t="str">
+      <c r="H3" t="str">
         <v/>
       </c>
     </row>
@@ -507,24 +496,21 @@
         <v>82</v>
       </c>
       <c r="C4" t="str">
-        <v>PRESTIMA SL Sucursal</v>
+        <v>FAA</v>
       </c>
       <c r="D4" t="str">
-        <v>FAA</v>
-      </c>
-      <c r="E4" t="str">
         <v>PECAS</v>
       </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
       <c r="F4">
-        <v>3</v>
+        <v>45</v>
       </c>
       <c r="G4">
-        <v>45</v>
-      </c>
-      <c r="H4">
         <v>5</v>
       </c>
-      <c r="I4" t="str">
+      <c r="H4" t="str">
         <v/>
       </c>
     </row>
@@ -536,30 +522,27 @@
         <v>100</v>
       </c>
       <c r="C5" t="str">
-        <v>Cliente Teste Lda</v>
+        <v>FR</v>
       </c>
       <c r="D5" t="str">
-        <v>FR</v>
-      </c>
-      <c r="E5" t="str">
         <v>SERV ADM</v>
       </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
       <c r="F5">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="G5">
-        <v>200</v>
-      </c>
-      <c r="H5">
         <v>0</v>
       </c>
-      <c r="I5" t="str">
+      <c r="H5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>